<commit_message>
AI+human review and edits
</commit_message>
<xml_diff>
--- a/release-notes/2026-06/closed-bugs-sle-2026-06.xlsx
+++ b/release-notes/2026-06/closed-bugs-sle-2026-06.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://emerson.sharepoint.com/sites/TM-IoTProgram/Shared Documents/ProjectDocuments/SystemLink 2026/2026 Q3 (v.26.5)(releasing out of Cycle 26.C2)/Common docs/26C2 Release Notes/SLE 2026-06 Release Notes/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/markblack/repos/install-systemlink-enterprise/release-notes/2026-06/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="384" documentId="8_{0357FC32-4DB0-FA47-B55E-60093BEFF741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9B6F4EF-2D96-487A-A91D-4C9AA5AE7DA2}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4928339-AC8A-594F-96D9-E48106D9EEC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13992" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="23240" windowHeight="14000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="closed bugs" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="12">
   <si>
     <t>ID</t>
   </si>
@@ -69,6 +69,9 @@
   </si>
   <si>
     <t>Work Items option is not visible in navigation bar despite having "Access work orders web application" privilege</t>
+  </si>
+  <si>
+    <t>Incorrect privilege validation when checking whether a system key can be rejected or deleted</t>
   </si>
 </sst>
 </file>
@@ -625,10 +628,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -928,15 +927,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.6"/>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.34765625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="119.59765625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.33203125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="119.6640625" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -947,7 +946,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>3860612</v>
       </c>
@@ -958,7 +957,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="3" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>3887214</v>
       </c>
@@ -969,7 +968,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="4" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>3887505</v>
       </c>
@@ -980,7 +979,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="5" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>3887507</v>
       </c>
@@ -991,7 +990,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="6" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>3889868</v>
       </c>
@@ -1002,7 +1001,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="7" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>3789353</v>
       </c>
@@ -1013,7 +1012,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="8" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>3835462</v>
       </c>
@@ -1021,6 +1020,17 @@
         <v>10</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="2">
+        <v>3780391</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1033,6 +1043,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CC68938C25E75A48B38E3943F7278D4C" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="47491c53f29c61f82c19f477ce8142ae">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="58dd0d8a-0b6e-4df8-afdb-fbe9bd3e42e9" xmlns:ns3="8f35f8fb-94b8-4296-88b5-253c68a5f93d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1234b2eb10b8f208397560529004cbac" ns2:_="" ns3:_="">
     <xsd:import namespace="58dd0d8a-0b6e-4df8-afdb-fbe9bd3e42e9"/>
@@ -1281,15 +1300,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1302,6 +1312,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8F5BA7BF-C649-45A8-BA98-72C6A48D6AFB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF8FE16A-F6E2-4383-A6A5-F239117A00DF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1316,14 +1334,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8F5BA7BF-C649-45A8-BA98-72C6A48D6AFB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>